<commit_message>
Add alt Tafel window analysis and fix overpotential decoupling plots
- Update Tafel regression window from [-3.5,-2.5] to [-3.5,-2.0] (alt set)
- Fix Tafel plot script to read from Edited/ subfolder (was reading BOL copies)
- Fix None-value filter in load_iv; add WINDOW_OVERRIDE support
- Update VC Polyol 30K slope to -0.0430 and AB BM 75K slope to -0.0489
- Add alt Tafel plots, kinetics Excel, and summary tables in tafel plot alt/
- Copy Overpotential DATA raw final to alt folder with updated S4/S5
- Add alt overpotential decoupling plots for all conditions and durabilities
- Fix colored bands clipping below I-V curve and fold-back bubble artifacts
- Add plot_overpotential_all_fixed.py, *_alt.py scripts for alt analysis

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/EIS/VC_BM_Transformed_Sets_15pct.xlsx
+++ b/EIS/VC_BM_Transformed_Sets_15pct.xlsx
@@ -432,22 +432,22 @@
         <v>-0.0593</v>
       </c>
       <c r="C2">
-        <v>0.05217314830495458</v>
+        <v>0.0521731483049545</v>
       </c>
       <c r="D2">
-        <v>-0.0593</v>
+        <v>-0.062858</v>
       </c>
       <c r="E2">
-        <v>0.04972662646220814</v>
+        <v>0.0497266264622081</v>
       </c>
       <c r="F2">
-        <v>-0.0593</v>
+        <v>-0.057521</v>
       </c>
       <c r="G2">
-        <v>0.05011304674111566</v>
+        <v>0.0501130467411156</v>
       </c>
       <c r="H2">
-        <v>-0.0593</v>
+        <v>-0.061079</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -458,22 +458,22 @@
         <v>-0.05395</v>
       </c>
       <c r="C3">
-        <v>0.05071166726735994</v>
+        <v>0.0507116672673599</v>
       </c>
       <c r="D3">
-        <v>-0.05395</v>
+        <v>-0.057187</v>
       </c>
       <c r="E3">
-        <v>0.04852683805953414</v>
+        <v>0.0485268380595341</v>
       </c>
       <c r="F3">
-        <v>-0.05395</v>
+        <v>-0.0523315</v>
       </c>
       <c r="G3">
-        <v>0.04887192482602119</v>
+        <v>0.0488719248260211</v>
       </c>
       <c r="H3">
-        <v>-0.05395</v>
+        <v>-0.0555685</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -484,22 +484,22 @@
         <v>-0.04899</v>
       </c>
       <c r="C4">
-        <v>0.04954474829935802</v>
+        <v>0.049544748299358</v>
       </c>
       <c r="D4">
-        <v>-0.04899</v>
+        <v>-0.0519294</v>
       </c>
       <c r="E4">
-        <v>0.04756886747445335</v>
+        <v>0.0475688674744533</v>
       </c>
       <c r="F4">
-        <v>-0.04899</v>
+        <v>-0.04752029999999999</v>
       </c>
       <c r="G4">
-        <v>0.04788095151396903</v>
+        <v>0.047880951513969</v>
       </c>
       <c r="H4">
-        <v>-0.04899</v>
+        <v>-0.0504597</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -510,22 +510,22 @@
         <v>-0.0445</v>
       </c>
       <c r="C5">
-        <v>0.04827586553803553</v>
+        <v>0.0482758655380355</v>
       </c>
       <c r="D5">
-        <v>-0.0445</v>
+        <v>-0.04717</v>
       </c>
       <c r="E5">
-        <v>0.04652719072174413</v>
+        <v>0.0465271907217441</v>
       </c>
       <c r="F5">
-        <v>-0.0445</v>
+        <v>-0.043165</v>
       </c>
       <c r="G5">
-        <v>0.04680338830086376</v>
+        <v>0.0468033883008637</v>
       </c>
       <c r="H5">
-        <v>-0.0445</v>
+        <v>-0.045835</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -536,22 +536,22 @@
         <v>-0.04053</v>
       </c>
       <c r="C6">
-        <v>0.04680305519007194</v>
+        <v>0.0468030551900719</v>
       </c>
       <c r="D6">
-        <v>-0.04053</v>
+        <v>-0.0429618</v>
       </c>
       <c r="E6">
-        <v>0.04531810163377808</v>
+        <v>0.045318101633778</v>
       </c>
       <c r="F6">
-        <v>-0.04053</v>
+        <v>-0.0393141</v>
       </c>
       <c r="G6">
         <v>0.0455526452856523</v>
       </c>
       <c r="H6">
-        <v>-0.04053</v>
+        <v>-0.0417459</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -562,22 +562,22 @@
         <v>-0.03665</v>
       </c>
       <c r="C7">
-        <v>0.04606665001609014</v>
+        <v>0.0460666500160901</v>
       </c>
       <c r="D7">
-        <v>-0.03665</v>
+        <v>-0.038849</v>
       </c>
       <c r="E7">
-        <v>0.04471355708979505</v>
+        <v>0.044713557089795</v>
       </c>
       <c r="F7">
-        <v>-0.03665</v>
+        <v>-0.0355505</v>
       </c>
       <c r="G7">
-        <v>0.04492727377804655</v>
+        <v>0.0449272737780465</v>
       </c>
       <c r="H7">
-        <v>-0.03665</v>
+        <v>-0.03774950000000001</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -588,22 +588,22 @@
         <v>-0.03307</v>
       </c>
       <c r="C8">
-        <v>0.04517163449694303</v>
+        <v>0.045171634496943</v>
       </c>
       <c r="D8">
-        <v>-0.03307</v>
+        <v>-0.0350542</v>
       </c>
       <c r="E8">
-        <v>0.04397880295172337</v>
+        <v>0.0439788029517233</v>
       </c>
       <c r="F8">
-        <v>-0.03307</v>
+        <v>-0.0320779</v>
       </c>
       <c r="G8">
-        <v>0.04416720686880266</v>
+        <v>0.0441672068688026</v>
       </c>
       <c r="H8">
-        <v>-0.03307</v>
+        <v>-0.0340621</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -614,22 +614,22 @@
         <v>-0.0299</v>
       </c>
       <c r="C9">
-        <v>0.04466181553034025</v>
+        <v>0.0446618155303402</v>
       </c>
       <c r="D9">
-        <v>-0.0299</v>
+        <v>-0.031694</v>
       </c>
       <c r="E9">
-        <v>0.04356027211358128</v>
+        <v>0.0435602721135812</v>
       </c>
       <c r="F9">
-        <v>-0.0299</v>
+        <v>-0.029003</v>
       </c>
       <c r="G9">
-        <v>0.04373425736353715</v>
+        <v>0.0437342573635371</v>
       </c>
       <c r="H9">
-        <v>-0.0299</v>
+        <v>-0.030797</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -640,22 +640,22 @@
         <v>-0.02712</v>
       </c>
       <c r="C10">
-        <v>0.04399338621857216</v>
+        <v>0.0439933862185721</v>
       </c>
       <c r="D10">
-        <v>-0.02712</v>
+        <v>-0.0287472</v>
       </c>
       <c r="E10">
-        <v>0.04301153168135053</v>
+        <v>0.0430115316813505</v>
       </c>
       <c r="F10">
-        <v>-0.02712</v>
+        <v>-0.0263064</v>
       </c>
       <c r="G10">
-        <v>0.04316661245663348</v>
+        <v>0.0431666124566334</v>
       </c>
       <c r="H10">
-        <v>-0.02712</v>
+        <v>-0.0279336</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -666,22 +666,22 @@
         <v>-0.02466</v>
       </c>
       <c r="C11">
-        <v>0.04349489656233832</v>
+        <v>0.0434948965623383</v>
       </c>
       <c r="D11">
-        <v>-0.02466</v>
+        <v>-0.0261396</v>
       </c>
       <c r="E11">
-        <v>0.04260230152850048</v>
+        <v>0.0426023015285004</v>
       </c>
       <c r="F11">
-        <v>-0.02466</v>
+        <v>-0.0239202</v>
       </c>
       <c r="G11">
-        <v>0.04274328405148498</v>
+        <v>0.0427432840514849</v>
       </c>
       <c r="H11">
-        <v>-0.02466</v>
+        <v>-0.0253998</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -692,22 +692,22 @@
         <v>-0.02244</v>
       </c>
       <c r="C12">
-        <v>0.04289444311278394</v>
+        <v>0.0428944431127839</v>
       </c>
       <c r="D12">
-        <v>-0.02244</v>
+        <v>-0.0237864</v>
       </c>
       <c r="E12">
-        <v>0.04210936520802202</v>
+        <v>0.042109365208022</v>
       </c>
       <c r="F12">
-        <v>-0.02244</v>
+        <v>-0.0217668</v>
       </c>
       <c r="G12">
-        <v>0.04223336574528339</v>
+        <v>0.0422333657452833</v>
       </c>
       <c r="H12">
-        <v>-0.02244</v>
+        <v>-0.0231132</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -721,19 +721,19 @@
         <v>0.042418612077288</v>
       </c>
       <c r="D13">
-        <v>-0.02041</v>
+        <v>-0.0216346</v>
       </c>
       <c r="E13">
-        <v>0.04171873642575606</v>
+        <v>0.041718736425756</v>
       </c>
       <c r="F13">
-        <v>-0.02041</v>
+        <v>-0.0197977</v>
       </c>
       <c r="G13">
-        <v>0.04182927954036891</v>
+        <v>0.0418292795403689</v>
       </c>
       <c r="H13">
-        <v>-0.02041</v>
+        <v>-0.0210223</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -744,22 +744,22 @@
         <v>-0.01858</v>
       </c>
       <c r="C14">
-        <v>0.04188613448994732</v>
+        <v>0.0418861344899473</v>
       </c>
       <c r="D14">
-        <v>-0.01858</v>
+        <v>-0.0196948</v>
       </c>
       <c r="E14">
-        <v>0.04128160421702987</v>
+        <v>0.0412816042170298</v>
       </c>
       <c r="F14">
-        <v>-0.01858</v>
+        <v>-0.0180226</v>
       </c>
       <c r="G14">
-        <v>0.04137708783486937</v>
+        <v>0.0413770878348693</v>
       </c>
       <c r="H14">
-        <v>-0.01858</v>
+        <v>-0.0191374</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -770,22 +770,22 @@
         <v>-0.01692</v>
       </c>
       <c r="C15">
-        <v>0.04137631552334454</v>
+        <v>0.0413763155233445</v>
       </c>
       <c r="D15">
-        <v>-0.01692</v>
+        <v>-0.0179352</v>
       </c>
       <c r="E15">
-        <v>0.04086307337888778</v>
+        <v>0.0408630733788877</v>
       </c>
       <c r="F15">
-        <v>-0.01692</v>
+        <v>-0.0164124</v>
       </c>
       <c r="G15">
-        <v>0.04094413832960386</v>
+        <v>0.0409441383296038</v>
       </c>
       <c r="H15">
-        <v>-0.01692</v>
+        <v>-0.0174276</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -796,22 +796,22 @@
         <v>-0.01533</v>
       </c>
       <c r="C16">
-        <v>0.04090048448784861</v>
+        <v>0.0409004844878486</v>
       </c>
       <c r="D16">
-        <v>-0.01533</v>
+        <v>-0.0162498</v>
       </c>
       <c r="E16">
-        <v>0.04047244459662182</v>
+        <v>0.0404724445966218</v>
       </c>
       <c r="F16">
-        <v>-0.01533</v>
+        <v>-0.0148701</v>
       </c>
       <c r="G16">
-        <v>0.04054005212468939</v>
+        <v>0.0405400521246893</v>
       </c>
       <c r="H16">
-        <v>-0.01533</v>
+        <v>-0.0157899</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -822,22 +822,22 @@
         <v>-0.01357</v>
       </c>
       <c r="C17">
-        <v>0.03977888276132248</v>
+        <v>0.0397788827613224</v>
       </c>
       <c r="D17">
-        <v>-0.01357</v>
+        <v>-0.0143842</v>
       </c>
       <c r="E17">
-        <v>0.03955167675270922</v>
+        <v>0.0395516767527092</v>
       </c>
       <c r="F17">
-        <v>-0.01357</v>
+        <v>-0.0131629</v>
       </c>
       <c r="G17">
-        <v>0.03958756321310527</v>
+        <v>0.0395875632131052</v>
       </c>
       <c r="H17">
-        <v>-0.01357</v>
+        <v>-0.0139771</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -848,22 +848,22 @@
         <v>-0.01218</v>
       </c>
       <c r="C18">
-        <v>0.03948432069172977</v>
+        <v>0.0394843206917297</v>
       </c>
       <c r="D18">
-        <v>-0.01218</v>
+        <v>-0.0129108</v>
       </c>
       <c r="E18">
-        <v>0.03930985893511601</v>
+        <v>0.039309858935116</v>
       </c>
       <c r="F18">
-        <v>-0.01218</v>
+        <v>-0.0118146</v>
       </c>
       <c r="G18">
-        <v>0.03933741461006297</v>
+        <v>0.0393374146100629</v>
       </c>
       <c r="H18">
-        <v>-0.01218</v>
+        <v>-0.0125454</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -874,22 +874,22 @@
         <v>-0.0109</v>
       </c>
       <c r="C19">
-        <v>0.03900848965623383</v>
+        <v>0.0390084896562338</v>
       </c>
       <c r="D19">
-        <v>-0.0109</v>
+        <v>-0.011554</v>
       </c>
       <c r="E19">
-        <v>0.03891923015285004</v>
+        <v>0.03891923015285</v>
       </c>
       <c r="F19">
-        <v>-0.0109</v>
+        <v>-0.010573</v>
       </c>
       <c r="G19">
-        <v>0.03893332840514849</v>
+        <v>0.0389333284051484</v>
       </c>
       <c r="H19">
-        <v>-0.0109</v>
+        <v>-0.011227</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -903,19 +903,19 @@
         <v>0.0386006344829516</v>
       </c>
       <c r="D20">
-        <v>-0.00954</v>
+        <v>-0.0101124</v>
       </c>
       <c r="E20">
-        <v>0.03858440548233637</v>
+        <v>0.0385844054823363</v>
       </c>
       <c r="F20">
-        <v>-0.00954</v>
+        <v>-0.0092538</v>
       </c>
       <c r="G20">
-        <v>0.03858696880093609</v>
+        <v>0.038586968800936</v>
       </c>
       <c r="H20">
-        <v>-0.00954</v>
+        <v>-0.0098262</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -929,19 +929,19 @@
         <v>0.03851</v>
       </c>
       <c r="D21">
-        <v>-0.00817</v>
+        <v>-0.0086602</v>
       </c>
       <c r="E21">
         <v>0.03851</v>
       </c>
       <c r="F21">
-        <v>-0.00817</v>
+        <v>-0.0079249</v>
       </c>
       <c r="G21">
         <v>0.03851</v>
       </c>
       <c r="H21">
-        <v>-0.00817</v>
+        <v>-0.0084151</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -952,22 +952,22 @@
         <v>-0.00714</v>
       </c>
       <c r="C22">
-        <v>0.03873658620737901</v>
+        <v>0.038736586207379</v>
       </c>
       <c r="D22">
-        <v>-0.00714</v>
+        <v>-0.0075684</v>
       </c>
       <c r="E22">
-        <v>0.03869601370584094</v>
+        <v>0.0386960137058409</v>
       </c>
       <c r="F22">
-        <v>-0.00714</v>
+        <v>-0.006925799999999999</v>
       </c>
       <c r="G22">
-        <v>0.03870242200234023</v>
+        <v>0.0387024220023402</v>
       </c>
       <c r="H22">
-        <v>-0.00714</v>
+        <v>-0.0073542</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -978,22 +978,22 @@
         <v>-0.00633</v>
       </c>
       <c r="C23">
-        <v>0.03879323275922377</v>
+        <v>0.0387932327592237</v>
       </c>
       <c r="D23">
-        <v>-0.00633</v>
+        <v>-0.0067098</v>
       </c>
       <c r="E23">
-        <v>0.03874251713230117</v>
+        <v>0.0387425171323011</v>
       </c>
       <c r="F23">
-        <v>-0.00633</v>
+        <v>-0.0061401</v>
       </c>
       <c r="G23">
-        <v>0.03875052750292528</v>
+        <v>0.0387505275029252</v>
       </c>
       <c r="H23">
-        <v>-0.00633</v>
+        <v>-0.006519899999999999</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1004,22 +1004,22 @@
         <v>-0.00561</v>
       </c>
       <c r="C24">
-        <v>0.03875924482811691</v>
+        <v>0.0387592448281169</v>
       </c>
       <c r="D24">
-        <v>-0.00561</v>
+        <v>-0.005946600000000001</v>
       </c>
       <c r="E24">
-        <v>0.03871461507642503</v>
+        <v>0.038714615076425</v>
       </c>
       <c r="F24">
-        <v>-0.00561</v>
+        <v>-0.0054417</v>
       </c>
       <c r="G24">
-        <v>0.03872166420257425</v>
+        <v>0.0387216642025742</v>
       </c>
       <c r="H24">
-        <v>-0.00561</v>
+        <v>-0.005778300000000001</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1030,22 +1030,22 @@
         <v>-0.00491</v>
       </c>
       <c r="C25">
-        <v>0.03867993965553426</v>
+        <v>0.0386799396555342</v>
       </c>
       <c r="D25">
-        <v>-0.00491</v>
+        <v>-0.0052046</v>
       </c>
       <c r="E25">
         <v>0.0386495102793807</v>
       </c>
       <c r="F25">
-        <v>-0.00491</v>
+        <v>-0.0047627</v>
       </c>
       <c r="G25">
-        <v>0.03865431650175517</v>
+        <v>0.0386543165017551</v>
       </c>
       <c r="H25">
-        <v>-0.00491</v>
+        <v>-0.005057300000000001</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -1059,19 +1059,19 @@
         <v>0.0386232931036895</v>
       </c>
       <c r="D26">
-        <v>-0.00424</v>
+        <v>-0.0044944</v>
       </c>
       <c r="E26">
-        <v>0.03860300685292047</v>
+        <v>0.0386030068529204</v>
       </c>
       <c r="F26">
-        <v>-0.00424</v>
+        <v>-0.0041128</v>
       </c>
       <c r="G26">
-        <v>0.03860621100117011</v>
+        <v>0.0386062110011701</v>
       </c>
       <c r="H26">
-        <v>-0.00424</v>
+        <v>-0.0043672</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -1082,22 +1082,22 @@
         <v>-0.00359</v>
       </c>
       <c r="C27">
-        <v>0.03856664655184475</v>
+        <v>0.0385666465518447</v>
       </c>
       <c r="D27">
-        <v>-0.00359</v>
+        <v>-0.0038054</v>
       </c>
       <c r="E27">
-        <v>0.03855650342646023</v>
+        <v>0.0385565034264602</v>
       </c>
       <c r="F27">
-        <v>-0.00359</v>
+        <v>-0.0034823</v>
       </c>
       <c r="G27">
-        <v>0.03855810550058505</v>
+        <v>0.038558105500585</v>
       </c>
       <c r="H27">
-        <v>-0.00359</v>
+        <v>-0.0036977</v>
       </c>
     </row>
     <row r="28" spans="1:8">
@@ -1111,19 +1111,19 @@
         <v>0.0386006344829516</v>
       </c>
       <c r="D28">
-        <v>-0.00303</v>
+        <v>-0.0032118</v>
       </c>
       <c r="E28">
-        <v>0.03858440548233637</v>
+        <v>0.0385844054823363</v>
       </c>
       <c r="F28">
-        <v>-0.00303</v>
+        <v>-0.0029391</v>
       </c>
       <c r="G28">
-        <v>0.03858696880093609</v>
+        <v>0.038586968800936</v>
       </c>
       <c r="H28">
-        <v>-0.00303</v>
+        <v>-0.0031209</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -1134,22 +1134,22 @@
         <v>-0.00244</v>
       </c>
       <c r="C29">
-        <v>0.03854398793110685</v>
+        <v>0.0385439879311068</v>
       </c>
       <c r="D29">
-        <v>-0.00244</v>
+        <v>-0.0025864</v>
       </c>
       <c r="E29">
-        <v>0.03853790205587614</v>
+        <v>0.0385379020558761</v>
       </c>
       <c r="F29">
-        <v>-0.00244</v>
+        <v>-0.0023668</v>
       </c>
       <c r="G29">
-        <v>0.03853886330035104</v>
+        <v>0.038538863300351</v>
       </c>
       <c r="H29">
-        <v>-0.00244</v>
+        <v>-0.0025132</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -1160,22 +1160,22 @@
         <v>-0.00188</v>
       </c>
       <c r="C30">
-        <v>0.03856664655184475</v>
+        <v>0.0385666465518447</v>
       </c>
       <c r="D30">
-        <v>-0.00188</v>
+        <v>-0.0019928</v>
       </c>
       <c r="E30">
-        <v>0.03855650342646023</v>
+        <v>0.0385565034264602</v>
       </c>
       <c r="F30">
-        <v>-0.00188</v>
+        <v>-0.0018236</v>
       </c>
       <c r="G30">
-        <v>0.03855810550058505</v>
+        <v>0.038558105500585</v>
       </c>
       <c r="H30">
-        <v>-0.00188</v>
+        <v>-0.0019364</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -1186,22 +1186,22 @@
         <v>-0.00135</v>
       </c>
       <c r="C31">
-        <v>0.03861196379332056</v>
+        <v>0.0386119637933205</v>
       </c>
       <c r="D31">
-        <v>-0.00135</v>
+        <v>-0.001431</v>
       </c>
       <c r="E31">
-        <v>0.03859370616762842</v>
+        <v>0.0385937061676284</v>
       </c>
       <c r="F31">
-        <v>-0.00135</v>
+        <v>-0.0013095</v>
       </c>
       <c r="G31">
-        <v>0.03859658990105311</v>
+        <v>0.0385965899010531</v>
       </c>
       <c r="H31">
-        <v>-0.00135</v>
+        <v>-0.0013905</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -1212,22 +1212,22 @@
         <v>-0.000865896</v>
       </c>
       <c r="C32">
-        <v>0.03866861034516531</v>
+        <v>0.0386686103451653</v>
       </c>
       <c r="D32">
-        <v>-0.000865896</v>
+        <v>-0.0009178497600000001</v>
       </c>
       <c r="E32">
-        <v>0.03864020959408865</v>
+        <v>0.0386402095940886</v>
       </c>
       <c r="F32">
-        <v>-0.000865896</v>
+        <v>-0.00083991912</v>
       </c>
       <c r="G32">
-        <v>0.03864469540163815</v>
+        <v>0.0386446954016381</v>
       </c>
       <c r="H32">
-        <v>-0.000865896</v>
+        <v>-0.00089187288</v>
       </c>
     </row>
     <row r="33" spans="1:8">
@@ -1238,22 +1238,22 @@
         <v>-0.000399365</v>
       </c>
       <c r="C33">
-        <v>0.03874791551774796</v>
+        <v>0.0387479155177479</v>
       </c>
       <c r="D33">
-        <v>-0.000399365</v>
+        <v>-0.0004233269</v>
       </c>
       <c r="E33">
-        <v>0.03870531439113298</v>
+        <v>0.0387053143911329</v>
       </c>
       <c r="F33">
-        <v>-0.000399365</v>
+        <v>-0.00038738405</v>
       </c>
       <c r="G33">
-        <v>0.03871204310245724</v>
+        <v>0.0387120431024572</v>
       </c>
       <c r="H33">
-        <v>-0.000399365</v>
+        <v>-0.00041134595</v>
       </c>
     </row>
     <row r="34" spans="1:8">
@@ -1264,22 +1264,22 @@
         <v>3.75269E-05</v>
       </c>
       <c r="C34">
-        <v>0.03883855000069957</v>
+        <v>0.0388385500006995</v>
       </c>
       <c r="D34">
-        <v>3.75269E-05</v>
+        <v>3.9778514E-05</v>
       </c>
       <c r="E34">
-        <v>0.03877971987346935</v>
+        <v>0.0387797198734693</v>
       </c>
       <c r="F34">
-        <v>3.75269E-05</v>
+        <v>3.6401093E-05</v>
       </c>
       <c r="G34">
-        <v>0.03878901190339333</v>
+        <v>0.0387890119033933</v>
       </c>
       <c r="H34">
-        <v>3.75269E-05</v>
+        <v>3.8652707E-05</v>
       </c>
     </row>
     <row r="35" spans="1:8">
@@ -1290,22 +1290,22 @@
         <v>0.000451407</v>
       </c>
       <c r="C35">
-        <v>0.03895184310438907</v>
+        <v>0.038951843104389</v>
       </c>
       <c r="D35">
-        <v>0.000451407</v>
+        <v>0.0004784914200000001</v>
       </c>
       <c r="E35">
-        <v>0.03887272672638981</v>
+        <v>0.0388727267263898</v>
       </c>
       <c r="F35">
-        <v>0.000451407</v>
+        <v>0.00043786479</v>
       </c>
       <c r="G35">
-        <v>0.03888522290456344</v>
+        <v>0.0388852229045634</v>
       </c>
       <c r="H35">
-        <v>0.000451407</v>
+        <v>0.00046494921</v>
       </c>
     </row>
     <row r="36" spans="1:8">
@@ -1316,22 +1316,22 @@
         <v>0.000848196</v>
       </c>
       <c r="C36">
-        <v>0.03908779482881648</v>
+        <v>0.0390877948288164</v>
       </c>
       <c r="D36">
-        <v>0.000848196</v>
+        <v>0.00089908776</v>
       </c>
       <c r="E36">
-        <v>0.03898433494989437</v>
+        <v>0.0389843349498943</v>
       </c>
       <c r="F36">
-        <v>0.000848196</v>
+        <v>0.00082275012</v>
       </c>
       <c r="G36">
-        <v>0.03900067610596758</v>
+        <v>0.0390006761059675</v>
       </c>
       <c r="H36">
-        <v>0.000848196</v>
+        <v>0.0008736418799999999</v>
       </c>
     </row>
     <row r="37" spans="1:8">
@@ -1345,19 +1345,19 @@
         <v>0.0392237465532439</v>
       </c>
       <c r="D37">
-        <v>0.00122</v>
+        <v>0.0012932</v>
       </c>
       <c r="E37">
-        <v>0.03909594317339894</v>
+        <v>0.0390959431733989</v>
       </c>
       <c r="F37">
-        <v>0.00122</v>
+        <v>0.0011834</v>
       </c>
       <c r="G37">
-        <v>0.03911612930737172</v>
+        <v>0.0391161293073717</v>
       </c>
       <c r="H37">
-        <v>0.00122</v>
+        <v>0.0012566</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -1368,22 +1368,22 @@
         <v>0.00158</v>
       </c>
       <c r="C38">
-        <v>0.03937102758804026</v>
+        <v>0.0393710275880402</v>
       </c>
       <c r="D38">
-        <v>0.00158</v>
+        <v>0.0016748</v>
       </c>
       <c r="E38">
-        <v>0.03921685208219554</v>
+        <v>0.0392168520821955</v>
       </c>
       <c r="F38">
-        <v>0.00158</v>
+        <v>0.0015326</v>
       </c>
       <c r="G38">
-        <v>0.03924120360889286</v>
+        <v>0.0392412036088928</v>
       </c>
       <c r="H38">
-        <v>0.00158</v>
+        <v>0.0016274</v>
       </c>
     </row>
     <row r="39" spans="1:8">
@@ -1394,22 +1394,22 @@
         <v>0.00193</v>
       </c>
       <c r="C39">
-        <v>0.03952963793320557</v>
+        <v>0.0395296379332055</v>
       </c>
       <c r="D39">
-        <v>0.00193</v>
+        <v>0.0020458</v>
       </c>
       <c r="E39">
-        <v>0.03934706167628419</v>
+        <v>0.0393470616762841</v>
       </c>
       <c r="F39">
-        <v>0.00193</v>
+        <v>0.0018721</v>
       </c>
       <c r="G39">
-        <v>0.03937589901053102</v>
+        <v>0.039375899010531</v>
       </c>
       <c r="H39">
-        <v>0.00193</v>
+        <v>0.0019879</v>
       </c>
     </row>
     <row r="40" spans="1:8">
@@ -1420,22 +1420,22 @@
         <v>0.00228</v>
       </c>
       <c r="C40">
-        <v>0.03967691896800193</v>
+        <v>0.0396769189680019</v>
       </c>
       <c r="D40">
-        <v>0.00228</v>
+        <v>0.0024168</v>
       </c>
       <c r="E40">
-        <v>0.03946797058508079</v>
+        <v>0.0394679705850807</v>
       </c>
       <c r="F40">
-        <v>0.00228</v>
+        <v>0.0022116</v>
       </c>
       <c r="G40">
-        <v>0.03950097331205216</v>
+        <v>0.0395009733120521</v>
       </c>
       <c r="H40">
-        <v>0.00228</v>
+        <v>0.0023484</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -1446,22 +1446,22 @@
         <v>0.00264</v>
       </c>
       <c r="C41">
-        <v>0.03982420000279828</v>
+        <v>0.0398242000027982</v>
       </c>
       <c r="D41">
-        <v>0.00264</v>
+        <v>0.0027984</v>
       </c>
       <c r="E41">
         <v>0.0395888794938774</v>
       </c>
       <c r="F41">
-        <v>0.00264</v>
+        <v>0.0025608</v>
       </c>
       <c r="G41">
-        <v>0.03962604761357331</v>
+        <v>0.0396260476135733</v>
       </c>
       <c r="H41">
-        <v>0.00264</v>
+        <v>0.0027192</v>
       </c>
     </row>
     <row r="42" spans="1:8">
@@ -1472,22 +1472,22 @@
         <v>0.00299</v>
       </c>
       <c r="C42">
-        <v>0.03997148103759465</v>
+        <v>0.0399714810375946</v>
       </c>
       <c r="D42">
-        <v>0.00299</v>
+        <v>0.0031694</v>
       </c>
       <c r="E42">
-        <v>0.03970978840267401</v>
+        <v>0.039709788402674</v>
       </c>
       <c r="F42">
-        <v>0.00299</v>
+        <v>0.0029003</v>
       </c>
       <c r="G42">
-        <v>0.03975112191509447</v>
+        <v>0.0397511219150944</v>
       </c>
       <c r="H42">
-        <v>0.00299</v>
+        <v>0.0030797</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -1498,22 +1498,22 @@
         <v>0.00336</v>
       </c>
       <c r="C43">
-        <v>0.04011876207239101</v>
+        <v>0.040118762072391</v>
       </c>
       <c r="D43">
-        <v>0.00336</v>
+        <v>0.0035616</v>
       </c>
       <c r="E43">
-        <v>0.03983069731147061</v>
+        <v>0.0398306973114706</v>
       </c>
       <c r="F43">
-        <v>0.00336</v>
+        <v>0.0032592</v>
       </c>
       <c r="G43">
-        <v>0.03987619621661561</v>
+        <v>0.0398761962166156</v>
       </c>
       <c r="H43">
-        <v>0.00336</v>
+        <v>0.0034608</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -1524,22 +1524,22 @@
         <v>0.00376</v>
       </c>
       <c r="C44">
-        <v>0.04026604310718736</v>
+        <v>0.0402660431071873</v>
       </c>
       <c r="D44">
-        <v>0.00376</v>
+        <v>0.0039856</v>
       </c>
       <c r="E44">
-        <v>0.03995160622026721</v>
+        <v>0.0399516062202672</v>
       </c>
       <c r="F44">
-        <v>0.00376</v>
+        <v>0.0036472</v>
       </c>
       <c r="G44">
-        <v>0.04000127051813675</v>
+        <v>0.0400012705181367</v>
       </c>
       <c r="H44">
-        <v>0.00376</v>
+        <v>0.0038728</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -1550,22 +1550,22 @@
         <v>0.00418</v>
       </c>
       <c r="C45">
-        <v>0.04040199483161477</v>
+        <v>0.0404019948316147</v>
       </c>
       <c r="D45">
-        <v>0.00418</v>
+        <v>0.004430799999999999</v>
       </c>
       <c r="E45">
-        <v>0.04006321444377178</v>
+        <v>0.0400632144437717</v>
       </c>
       <c r="F45">
-        <v>0.00418</v>
+        <v>0.004054599999999999</v>
       </c>
       <c r="G45">
-        <v>0.04011672371954089</v>
+        <v>0.0401167237195408</v>
       </c>
       <c r="H45">
-        <v>0.00418</v>
+        <v>0.0043054</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -1576,22 +1576,22 @@
         <v>0.00463</v>
       </c>
       <c r="C46">
-        <v>0.04053794655604218</v>
+        <v>0.0405379465560421</v>
       </c>
       <c r="D46">
-        <v>0.00463</v>
+        <v>0.004907799999999999</v>
       </c>
       <c r="E46">
-        <v>0.04017482266727634</v>
+        <v>0.0401748226672763</v>
       </c>
       <c r="F46">
-        <v>0.00463</v>
+        <v>0.0044911</v>
       </c>
       <c r="G46">
-        <v>0.04023217692094503</v>
+        <v>0.040232176920945</v>
       </c>
       <c r="H46">
-        <v>0.00463</v>
+        <v>0.0047689</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -1602,22 +1602,22 @@
         <v>0.00513</v>
       </c>
       <c r="C47">
-        <v>0.04066256897010064</v>
+        <v>0.0406625689701006</v>
       </c>
       <c r="D47">
-        <v>0.00513</v>
+        <v>0.0054378</v>
       </c>
       <c r="E47">
-        <v>0.04027713020548885</v>
+        <v>0.0402771302054888</v>
       </c>
       <c r="F47">
-        <v>0.00513</v>
+        <v>0.0049761</v>
       </c>
       <c r="G47">
-        <v>0.04033800902223215</v>
+        <v>0.0403380090222321</v>
       </c>
       <c r="H47">
-        <v>0.00513</v>
+        <v>0.0052839</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -1628,22 +1628,22 @@
         <v>0.00567</v>
       </c>
       <c r="C48">
-        <v>0.04079852069452804</v>
+        <v>0.040798520694528</v>
       </c>
       <c r="D48">
-        <v>0.00567</v>
+        <v>0.0060102</v>
       </c>
       <c r="E48">
         <v>0.0403887384289934</v>
       </c>
       <c r="F48">
-        <v>0.00567</v>
+        <v>0.005499899999999999</v>
       </c>
       <c r="G48">
-        <v>0.04045346222363629</v>
+        <v>0.0404534622236362</v>
       </c>
       <c r="H48">
-        <v>0.00567</v>
+        <v>0.0058401</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -1654,22 +1654,22 @@
         <v>0.00627</v>
       </c>
       <c r="C49">
-        <v>0.04093447241895545</v>
+        <v>0.0409344724189554</v>
       </c>
       <c r="D49">
-        <v>0.00627</v>
+        <v>0.006646200000000001</v>
       </c>
       <c r="E49">
-        <v>0.04050034665249796</v>
+        <v>0.0405003466524979</v>
       </c>
       <c r="F49">
-        <v>0.00627</v>
+        <v>0.0060819</v>
       </c>
       <c r="G49">
-        <v>0.04056891542504042</v>
+        <v>0.0405689154250404</v>
       </c>
       <c r="H49">
-        <v>0.00627</v>
+        <v>0.0064581</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -1680,22 +1680,22 @@
         <v>0.00694</v>
       </c>
       <c r="C50">
-        <v>0.04107042414338287</v>
+        <v>0.0410704241433828</v>
       </c>
       <c r="D50">
-        <v>0.00694</v>
+        <v>0.007356400000000001</v>
       </c>
       <c r="E50">
-        <v>0.04061195487600252</v>
+        <v>0.0406119548760025</v>
       </c>
       <c r="F50">
-        <v>0.00694</v>
+        <v>0.0067318</v>
       </c>
       <c r="G50">
-        <v>0.04068436862644456</v>
+        <v>0.0406843686264445</v>
       </c>
       <c r="H50">
-        <v>0.00694</v>
+        <v>0.0071482</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -1706,22 +1706,22 @@
         <v>0.00768</v>
       </c>
       <c r="C51">
-        <v>0.04120637586781028</v>
+        <v>0.0412063758678102</v>
       </c>
       <c r="D51">
-        <v>0.00768</v>
+        <v>0.0081408</v>
       </c>
       <c r="E51">
-        <v>0.04072356309950708</v>
+        <v>0.040723563099507</v>
       </c>
       <c r="F51">
-        <v>0.00768</v>
+        <v>0.0074496</v>
       </c>
       <c r="G51">
         <v>0.0407998218278487</v>
       </c>
       <c r="H51">
-        <v>0.00768</v>
+        <v>0.0079104</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -1732,22 +1732,22 @@
         <v>0.008500000000000001</v>
       </c>
       <c r="C52">
-        <v>0.04134232759223768</v>
+        <v>0.0413423275922376</v>
       </c>
       <c r="D52">
-        <v>0.008500000000000001</v>
+        <v>0.009010000000000001</v>
       </c>
       <c r="E52">
-        <v>0.04083517132301163</v>
+        <v>0.0408351713230116</v>
       </c>
       <c r="F52">
-        <v>0.008500000000000001</v>
+        <v>0.008245000000000001</v>
       </c>
       <c r="G52">
-        <v>0.04091527502925283</v>
+        <v>0.0409152750292528</v>
       </c>
       <c r="H52">
-        <v>0.008500000000000001</v>
+        <v>0.008755000000000001</v>
       </c>
     </row>
     <row r="53" spans="1:8">
@@ -1758,22 +1758,22 @@
         <v>0.00942</v>
       </c>
       <c r="C53">
-        <v>0.04148960862703405</v>
+        <v>0.041489608627034</v>
       </c>
       <c r="D53">
-        <v>0.00942</v>
+        <v>0.0099852</v>
       </c>
       <c r="E53">
-        <v>0.04095608023180825</v>
+        <v>0.0409560802318082</v>
       </c>
       <c r="F53">
-        <v>0.00942</v>
+        <v>0.009137399999999999</v>
       </c>
       <c r="G53">
-        <v>0.04104034933077398</v>
+        <v>0.0410403493307739</v>
       </c>
       <c r="H53">
-        <v>0.00942</v>
+        <v>0.0097026</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -1784,22 +1784,22 @@
         <v>0.01044</v>
       </c>
       <c r="C54">
-        <v>0.04164821897219935</v>
+        <v>0.0416482189721993</v>
       </c>
       <c r="D54">
-        <v>0.01044</v>
+        <v>0.0110664</v>
       </c>
       <c r="E54">
-        <v>0.04108628982589689</v>
+        <v>0.0410862898258968</v>
       </c>
       <c r="F54">
-        <v>0.01044</v>
+        <v>0.0101268</v>
       </c>
       <c r="G54">
-        <v>0.04117504473241213</v>
+        <v>0.0411750447324121</v>
       </c>
       <c r="H54">
-        <v>0.01044</v>
+        <v>0.0107532</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -1810,22 +1810,22 @@
         <v>0.01158</v>
       </c>
       <c r="C55">
-        <v>0.04181815862773362</v>
+        <v>0.0418181586277336</v>
       </c>
       <c r="D55">
-        <v>0.01158</v>
+        <v>0.0122748</v>
       </c>
       <c r="E55">
         <v>0.0412258001052776</v>
       </c>
       <c r="F55">
-        <v>0.01158</v>
+        <v>0.0112326</v>
       </c>
       <c r="G55">
-        <v>0.04131936123416731</v>
+        <v>0.0413193612341673</v>
       </c>
       <c r="H55">
-        <v>0.01158</v>
+        <v>0.0119274</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -1836,22 +1836,22 @@
         <v>0.01285</v>
       </c>
       <c r="C56">
-        <v>0.04201075690400578</v>
+        <v>0.0420107569040057</v>
       </c>
       <c r="D56">
-        <v>0.01285</v>
+        <v>0.013621</v>
       </c>
       <c r="E56">
-        <v>0.04138391175524238</v>
+        <v>0.0413839117552423</v>
       </c>
       <c r="F56">
-        <v>0.01285</v>
+        <v>0.0124645</v>
       </c>
       <c r="G56">
         <v>0.0414829199361565</v>
       </c>
       <c r="H56">
-        <v>0.01285</v>
+        <v>0.0132355</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -1862,22 +1862,22 @@
         <v>0.01426</v>
       </c>
       <c r="C57">
-        <v>0.04220335518027794</v>
+        <v>0.0422033551802779</v>
       </c>
       <c r="D57">
-        <v>0.01426</v>
+        <v>0.0151156</v>
       </c>
       <c r="E57">
-        <v>0.04154202340520718</v>
+        <v>0.0415420234052071</v>
       </c>
       <c r="F57">
-        <v>0.01426</v>
+        <v>0.0138322</v>
       </c>
       <c r="G57">
         <v>0.0416464786381457</v>
       </c>
       <c r="H57">
-        <v>0.01426</v>
+        <v>0.0146878</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -1891,19 +1891,19 @@
         <v>0.042418612077288</v>
       </c>
       <c r="D58">
-        <v>0.01584</v>
+        <v>0.0167904</v>
       </c>
       <c r="E58">
-        <v>0.04171873642575606</v>
+        <v>0.041718736425756</v>
       </c>
       <c r="F58">
-        <v>0.01584</v>
+        <v>0.0153648</v>
       </c>
       <c r="G58">
-        <v>0.04182927954036891</v>
+        <v>0.0418292795403689</v>
       </c>
       <c r="H58">
-        <v>0.01584</v>
+        <v>0.0163152</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -1914,22 +1914,22 @@
         <v>0.0176</v>
       </c>
       <c r="C59">
-        <v>0.04265652759503596</v>
+        <v>0.0426565275950359</v>
       </c>
       <c r="D59">
-        <v>0.0176</v>
+        <v>0.018656</v>
       </c>
       <c r="E59">
-        <v>0.04191405081688904</v>
+        <v>0.041914050816889</v>
       </c>
       <c r="F59">
-        <v>0.0176</v>
+        <v>0.017072</v>
       </c>
       <c r="G59">
-        <v>0.04203132264282614</v>
+        <v>0.0420313226428261</v>
       </c>
       <c r="H59">
-        <v>0.0176</v>
+        <v>0.018128</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -1940,22 +1940,22 @@
         <v>0.01956</v>
       </c>
       <c r="C60">
-        <v>0.04290577242315288</v>
+        <v>0.0429057724231528</v>
       </c>
       <c r="D60">
-        <v>0.01956</v>
+        <v>0.0207336</v>
       </c>
       <c r="E60">
-        <v>0.04211866589331406</v>
+        <v>0.042118665893314</v>
       </c>
       <c r="F60">
-        <v>0.01956</v>
+        <v>0.0189732</v>
       </c>
       <c r="G60">
-        <v>0.04224298684540039</v>
+        <v>0.0422429868454003</v>
       </c>
       <c r="H60">
-        <v>0.01956</v>
+        <v>0.0201468</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -1969,19 +1969,19 @@
         <v>0.0432003344927456</v>
       </c>
       <c r="D61">
-        <v>0.02175</v>
+        <v>0.023055</v>
       </c>
       <c r="E61">
-        <v>0.04236048371090727</v>
+        <v>0.0423604837109072</v>
       </c>
       <c r="F61">
-        <v>0.02175</v>
+        <v>0.0210975</v>
       </c>
       <c r="G61">
-        <v>0.04249313544844269</v>
+        <v>0.0424931354484426</v>
       </c>
       <c r="H61">
-        <v>0.02175</v>
+        <v>0.0224025</v>
       </c>
     </row>
     <row r="62" spans="1:8">
@@ -1992,22 +1992,22 @@
         <v>0.02419</v>
       </c>
       <c r="C62">
-        <v>0.04352888449344518</v>
+        <v>0.0435288844934451</v>
       </c>
       <c r="D62">
-        <v>0.02419</v>
+        <v>0.0256414</v>
       </c>
       <c r="E62">
-        <v>0.04263020358437662</v>
+        <v>0.0426302035843766</v>
       </c>
       <c r="F62">
-        <v>0.02419</v>
+        <v>0.0234643</v>
       </c>
       <c r="G62">
-        <v>0.04277214735183602</v>
+        <v>0.042772147351836</v>
       </c>
       <c r="H62">
-        <v>0.02419</v>
+        <v>0.0249157</v>
       </c>
     </row>
     <row r="63" spans="1:8">
@@ -2018,22 +2018,22 @@
         <v>0.0269</v>
       </c>
       <c r="C63">
-        <v>0.04388009311488265</v>
+        <v>0.0438800931148826</v>
       </c>
       <c r="D63">
-        <v>0.0269</v>
+        <v>0.028514</v>
       </c>
       <c r="E63">
-        <v>0.04291852482843006</v>
+        <v>0.04291852482843</v>
       </c>
       <c r="F63">
-        <v>0.0269</v>
+        <v>0.026093</v>
       </c>
       <c r="G63">
-        <v>0.04307040145546336</v>
+        <v>0.0430704014554633</v>
       </c>
       <c r="H63">
-        <v>0.0269</v>
+        <v>0.027707</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2044,22 +2044,22 @@
         <v>0.02993</v>
       </c>
       <c r="C64">
-        <v>0.04427661897779592</v>
+        <v>0.0442766189777959</v>
       </c>
       <c r="D64">
-        <v>0.02993</v>
+        <v>0.0317258</v>
       </c>
       <c r="E64">
-        <v>0.04324404881365169</v>
+        <v>0.0432440488136516</v>
       </c>
       <c r="F64">
-        <v>0.02993</v>
+        <v>0.0290321</v>
       </c>
       <c r="G64">
-        <v>0.04340713995955876</v>
+        <v>0.0434071399595587</v>
       </c>
       <c r="H64">
-        <v>0.02993</v>
+        <v>0.0308279</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2070,22 +2070,22 @@
         <v>0.0333</v>
       </c>
       <c r="C65">
-        <v>0.04472979139255395</v>
+        <v>0.0447297913925539</v>
       </c>
       <c r="D65">
-        <v>0.0333</v>
+        <v>0.035298</v>
       </c>
       <c r="E65">
-        <v>0.04361607622533355</v>
+        <v>0.0436160762253335</v>
       </c>
       <c r="F65">
-        <v>0.0333</v>
+        <v>0.032301</v>
       </c>
       <c r="G65">
-        <v>0.04379198396423922</v>
+        <v>0.0437919839642392</v>
       </c>
       <c r="H65">
-        <v>0.0333</v>
+        <v>0.034299</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2096,22 +2096,22 @@
         <v>0.03706</v>
       </c>
       <c r="C66">
-        <v>0.04523961035915674</v>
+        <v>0.0452396103591567</v>
       </c>
       <c r="D66">
-        <v>0.03706</v>
+        <v>0.0392836</v>
       </c>
       <c r="E66">
-        <v>0.04403460706347566</v>
+        <v>0.0440346070634756</v>
       </c>
       <c r="F66">
-        <v>0.03706</v>
+        <v>0.0359482</v>
       </c>
       <c r="G66">
-        <v>0.04422493346950473</v>
+        <v>0.0442249334695047</v>
       </c>
       <c r="H66">
-        <v>0.03706</v>
+        <v>0.03817180000000001</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -2122,22 +2122,22 @@
         <v>0.04124</v>
       </c>
       <c r="C67">
-        <v>0.04580607587760427</v>
+        <v>0.0458060758776042</v>
       </c>
       <c r="D67">
-        <v>0.04124</v>
+        <v>0.0437144</v>
       </c>
       <c r="E67">
-        <v>0.04449964132807798</v>
+        <v>0.0444996413280779</v>
       </c>
       <c r="F67">
-        <v>0.04124</v>
+        <v>0.0400028</v>
       </c>
       <c r="G67">
-        <v>0.04470598847535529</v>
+        <v>0.0447059884753552</v>
       </c>
       <c r="H67">
-        <v>0.04124</v>
+        <v>0.0424772</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -2148,22 +2148,22 @@
         <v>0.04589</v>
       </c>
       <c r="C68">
-        <v>0.04644051725826552</v>
+        <v>0.0464405172582655</v>
       </c>
       <c r="D68">
-        <v>0.04589</v>
+        <v>0.0486434</v>
       </c>
       <c r="E68">
-        <v>0.04502047970443259</v>
+        <v>0.0450204797044325</v>
       </c>
       <c r="F68">
-        <v>0.04589</v>
+        <v>0.0445133</v>
       </c>
       <c r="G68">
-        <v>0.04524477008190793</v>
+        <v>0.0452447700819079</v>
       </c>
       <c r="H68">
-        <v>0.04589</v>
+        <v>0.0472667</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2174,22 +2174,22 @@
         <v>0.05106</v>
       </c>
       <c r="C69">
-        <v>0.04717692243224731</v>
+        <v>0.0471769224322473</v>
       </c>
       <c r="D69">
-        <v>0.05106</v>
+        <v>0.0541236</v>
       </c>
       <c r="E69">
-        <v>0.04562502424841561</v>
+        <v>0.0456250242484156</v>
       </c>
       <c r="F69">
-        <v>0.05106</v>
+        <v>0.0495282</v>
       </c>
       <c r="G69">
-        <v>0.04587014158951366</v>
+        <v>0.0458701415895136</v>
       </c>
       <c r="H69">
-        <v>0.05106</v>
+        <v>0.0525918</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2200,22 +2200,22 @@
         <v>0.05683</v>
       </c>
       <c r="C70">
-        <v>0.04798130346844282</v>
+        <v>0.0479813034684428</v>
       </c>
       <c r="D70">
-        <v>0.05683</v>
+        <v>0.0602398</v>
       </c>
       <c r="E70">
-        <v>0.04628537290415092</v>
+        <v>0.0462853729041509</v>
       </c>
       <c r="F70">
-        <v>0.05683</v>
+        <v>0.0551251</v>
       </c>
       <c r="G70">
-        <v>0.04655323969782147</v>
+        <v>0.0465532396978214</v>
       </c>
       <c r="H70">
-        <v>0.05683</v>
+        <v>0.0585349</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2226,22 +2226,22 @@
         <v>0.06324</v>
       </c>
       <c r="C71">
-        <v>0.04888764829795887</v>
+        <v>0.0488876482979588</v>
       </c>
       <c r="D71">
-        <v>0.06324</v>
+        <v>0.06703440000000001</v>
       </c>
       <c r="E71">
-        <v>0.04702942772751464</v>
+        <v>0.0470294277275146</v>
       </c>
       <c r="F71">
-        <v>0.06324</v>
+        <v>0.0613428</v>
       </c>
       <c r="G71">
-        <v>0.04732292770718237</v>
+        <v>0.0473229277071823</v>
       </c>
       <c r="H71">
-        <v>0.06324</v>
+        <v>0.06513720000000001</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2252,22 +2252,22 @@
         <v>0.07037</v>
       </c>
       <c r="C72">
-        <v>0.04992994485190234</v>
+        <v>0.0499299448519023</v>
       </c>
       <c r="D72">
-        <v>0.07037</v>
+        <v>0.07459220000000001</v>
       </c>
       <c r="E72">
-        <v>0.04788509077438292</v>
+        <v>0.0478850907743829</v>
       </c>
       <c r="F72">
-        <v>0.07037</v>
+        <v>0.0682589</v>
       </c>
       <c r="G72">
-        <v>0.04820806891794742</v>
+        <v>0.0482080689179474</v>
       </c>
       <c r="H72">
-        <v>0.07037</v>
+        <v>0.07248110000000001</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2278,22 +2278,22 @@
         <v>0.07828</v>
       </c>
       <c r="C73">
-        <v>0.05107420519916636</v>
+        <v>0.0510742051991663</v>
       </c>
       <c r="D73">
-        <v>0.07828</v>
+        <v>0.0829768</v>
       </c>
       <c r="E73">
-        <v>0.04882445998887963</v>
+        <v>0.0488244599888796</v>
       </c>
       <c r="F73">
-        <v>0.07828</v>
+        <v>0.0759316</v>
       </c>
       <c r="G73">
-        <v>0.04917980002976556</v>
+        <v>0.0491798000297655</v>
       </c>
       <c r="H73">
-        <v>0.07828</v>
+        <v>0.0806284</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -2307,19 +2307,19 @@
         <v>0.0523770758915957</v>
       </c>
       <c r="D74">
-        <v>0.08709</v>
+        <v>0.09231540000000001</v>
       </c>
       <c r="E74">
-        <v>0.04989403879746498</v>
+        <v>0.0498940387974649</v>
       </c>
       <c r="F74">
-        <v>0.08709</v>
+        <v>0.08447730000000001</v>
       </c>
       <c r="G74">
-        <v>0.05028622654322187</v>
+        <v>0.0502862265432218</v>
       </c>
       <c r="H74">
-        <v>0.08709</v>
+        <v>0.0897027</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -2330,22 +2330,22 @@
         <v>0.09687</v>
       </c>
       <c r="C75">
-        <v>0.05383855692919035</v>
+        <v>0.0538385569291903</v>
       </c>
       <c r="D75">
-        <v>0.09687</v>
+        <v>0.1026822</v>
       </c>
       <c r="E75">
-        <v>0.05109382720013899</v>
+        <v>0.0510938272001389</v>
       </c>
       <c r="F75">
-        <v>0.09687</v>
+        <v>0.09396389999999999</v>
       </c>
       <c r="G75">
-        <v>0.05152734845831633</v>
+        <v>0.0515273484583163</v>
       </c>
       <c r="H75">
-        <v>0.09687</v>
+        <v>0.09977610000000001</v>
       </c>
     </row>
     <row r="76" spans="1:8">
@@ -2356,22 +2356,22 @@
         <v>0.10776</v>
       </c>
       <c r="C76">
-        <v>0.05549263624305716</v>
+        <v>0.0554926362430571</v>
       </c>
       <c r="D76">
-        <v>0.10776</v>
+        <v>0.1142256</v>
       </c>
       <c r="E76">
-        <v>0.05245172725277779</v>
+        <v>0.0524517272527777</v>
       </c>
       <c r="F76">
-        <v>0.10776</v>
+        <v>0.1045272</v>
       </c>
       <c r="G76">
-        <v>0.05293202907539998</v>
+        <v>0.0529320290753999</v>
       </c>
       <c r="H76">
-        <v>0.10776</v>
+        <v>0.1109928</v>
       </c>
     </row>
     <row r="77" spans="1:8">
@@ -2382,22 +2382,22 @@
         <v>0.11982</v>
       </c>
       <c r="C77">
-        <v>0.05731665521245822</v>
+        <v>0.0573166552124582</v>
       </c>
       <c r="D77">
-        <v>0.11982</v>
+        <v>0.1270092</v>
       </c>
       <c r="E77">
-        <v>0.05394913758479728</v>
+        <v>0.0539491375847972</v>
       </c>
       <c r="F77">
-        <v>0.11982</v>
+        <v>0.1162254</v>
       </c>
       <c r="G77">
         <v>0.0544810261942388</v>
       </c>
       <c r="H77">
-        <v>0.11982</v>
+        <v>0.1234146</v>
       </c>
     </row>
     <row r="78" spans="1:8">
@@ -2408,22 +2408,22 @@
         <v>0.13323</v>
       </c>
       <c r="C78">
-        <v>0.05940124832034516</v>
+        <v>0.0594012483203451</v>
       </c>
       <c r="D78">
-        <v>0.13323</v>
+        <v>0.1412238</v>
       </c>
       <c r="E78">
-        <v>0.05566046367853385</v>
+        <v>0.0556604636785338</v>
       </c>
       <c r="F78">
-        <v>0.13323</v>
+        <v>0.1292331</v>
       </c>
       <c r="G78">
-        <v>0.05625130861576888</v>
+        <v>0.0562513086157688</v>
       </c>
       <c r="H78">
-        <v>0.13323</v>
+        <v>0.1372269</v>
       </c>
     </row>
     <row r="79" spans="1:8">
@@ -2434,22 +2434,22 @@
         <v>0.14812</v>
       </c>
       <c r="C79">
-        <v>0.06173508625634901</v>
+        <v>0.061735086256349</v>
       </c>
       <c r="D79">
-        <v>0.14812</v>
+        <v>0.1570072</v>
       </c>
       <c r="E79">
-        <v>0.05757640484869544</v>
+        <v>0.0575764048486954</v>
       </c>
       <c r="F79">
-        <v>0.14812</v>
+        <v>0.1436764</v>
       </c>
       <c r="G79">
-        <v>0.05823325523987322</v>
+        <v>0.0582332552398732</v>
       </c>
       <c r="H79">
-        <v>0.14812</v>
+        <v>0.1525636</v>
       </c>
     </row>
     <row r="80" spans="1:8">
@@ -2460,22 +2460,22 @@
         <v>0.16481</v>
       </c>
       <c r="C80">
-        <v>0.06431816902046977</v>
+        <v>0.0643181690204697</v>
       </c>
       <c r="D80">
-        <v>0.16481</v>
+        <v>0.1746986</v>
       </c>
       <c r="E80">
-        <v>0.05969696109528205</v>
+        <v>0.059696961095282</v>
       </c>
       <c r="F80">
-        <v>0.16481</v>
+        <v>0.1598657</v>
       </c>
       <c r="G80">
         <v>0.0604268660665518</v>
       </c>
       <c r="H80">
-        <v>0.16481</v>
+        <v>0.1697543</v>
       </c>
     </row>
     <row r="81" spans="1:8">
@@ -2489,19 +2489,19 @@
         <v>0.0672071431645522</v>
       </c>
       <c r="D81">
-        <v>0.18318</v>
+        <v>0.1941708</v>
       </c>
       <c r="E81">
-        <v>0.06206863584475392</v>
+        <v>0.0620686358447539</v>
       </c>
       <c r="F81">
-        <v>0.18318</v>
+        <v>0.1776846</v>
       </c>
       <c r="G81">
-        <v>0.06288024659638969</v>
+        <v>0.06288024659638961</v>
       </c>
       <c r="H81">
-        <v>0.18318</v>
+        <v>0.1886754</v>
       </c>
     </row>
     <row r="82" spans="1:8">
@@ -2512,22 +2512,22 @@
         <v>0.20356</v>
       </c>
       <c r="C82">
-        <v>0.07036802075748946</v>
+        <v>0.07036802075748939</v>
       </c>
       <c r="D82">
-        <v>0.20356</v>
+        <v>0.2157736</v>
       </c>
       <c r="E82">
         <v>0.0646635270412349</v>
       </c>
       <c r="F82">
-        <v>0.20356</v>
+        <v>0.1974532</v>
       </c>
       <c r="G82">
-        <v>0.06556453352903584</v>
+        <v>0.0655645335290358</v>
       </c>
       <c r="H82">
-        <v>0.20356</v>
+        <v>0.2096668</v>
       </c>
     </row>
     <row r="83" spans="1:8">
@@ -2538,22 +2538,22 @@
         <v>0.22619</v>
       </c>
       <c r="C83">
-        <v>0.07394808283407792</v>
+        <v>0.0739480828340779</v>
       </c>
       <c r="D83">
-        <v>0.22619</v>
+        <v>0.2397614</v>
       </c>
       <c r="E83">
-        <v>0.06760254359352162</v>
+        <v>0.06760254359352159</v>
       </c>
       <c r="F83">
-        <v>0.22619</v>
+        <v>0.2194043</v>
       </c>
       <c r="G83">
-        <v>0.06860480116601143</v>
+        <v>0.06860480116601141</v>
       </c>
       <c r="H83">
-        <v>0.22619</v>
+        <v>0.2329757</v>
       </c>
     </row>
     <row r="84" spans="1:8">
@@ -2567,19 +2567,19 @@
         <v>0.0779020121528417</v>
       </c>
       <c r="D84">
-        <v>0.25132</v>
+        <v>0.2663992</v>
       </c>
       <c r="E84">
-        <v>0.07084848276044586</v>
+        <v>0.07084848276044579</v>
       </c>
       <c r="F84">
-        <v>0.25132</v>
+        <v>0.2437804</v>
       </c>
       <c r="G84">
-        <v>0.07196256510684837</v>
+        <v>0.0719625651068483</v>
       </c>
       <c r="H84">
-        <v>0.25132</v>
+        <v>0.2588596</v>
       </c>
     </row>
     <row r="85" spans="1:8">
@@ -2590,22 +2590,22 @@
         <v>0.27917</v>
       </c>
       <c r="C85">
-        <v>0.08219582078267404</v>
+        <v>0.082195820782674</v>
       </c>
       <c r="D85">
-        <v>0.27917</v>
+        <v>0.2959202</v>
       </c>
       <c r="E85">
-        <v>0.07437344248613151</v>
+        <v>0.07437344248613149</v>
       </c>
       <c r="F85">
-        <v>0.27917</v>
+        <v>0.2707948999999999</v>
       </c>
       <c r="G85">
-        <v>0.07560896205119566</v>
+        <v>0.07560896205119561</v>
       </c>
       <c r="H85">
-        <v>0.27917</v>
+        <v>0.2875451</v>
       </c>
     </row>
     <row r="86" spans="1:8">
@@ -2616,22 +2616,22 @@
         <v>0.3101</v>
       </c>
       <c r="C86">
-        <v>0.08688615527541965</v>
+        <v>0.0868861552754196</v>
       </c>
       <c r="D86">
-        <v>0.3101</v>
+        <v>0.328706</v>
       </c>
       <c r="E86">
         <v>0.0782239261970388</v>
       </c>
       <c r="F86">
-        <v>0.3101</v>
+        <v>0.300797</v>
       </c>
       <c r="G86">
-        <v>0.07959209749963836</v>
+        <v>0.0795920974996383</v>
       </c>
       <c r="H86">
-        <v>0.3101</v>
+        <v>0.319403</v>
       </c>
     </row>
     <row r="87" spans="1:8">
@@ -2642,22 +2642,22 @@
         <v>0.34461</v>
       </c>
       <c r="C87">
-        <v>0.09239220011472969</v>
+        <v>0.09239220011472959</v>
       </c>
       <c r="D87">
-        <v>0.34461</v>
+        <v>0.3652866000000001</v>
       </c>
       <c r="E87">
         <v>0.08274405924897341</v>
       </c>
       <c r="F87">
-        <v>0.34461</v>
+        <v>0.3342717</v>
       </c>
       <c r="G87">
-        <v>0.08426795215650586</v>
+        <v>0.0842679521565058</v>
       </c>
       <c r="H87">
-        <v>0.34461</v>
+        <v>0.3549483</v>
       </c>
     </row>
     <row r="88" spans="1:8">
@@ -2668,22 +2668,22 @@
         <v>0.38232</v>
       </c>
       <c r="C88">
-        <v>0.09778495185035024</v>
+        <v>0.0977849518503502</v>
       </c>
       <c r="D88">
-        <v>0.38232</v>
+        <v>0.4052592</v>
       </c>
       <c r="E88">
-        <v>0.08717118544798758</v>
+        <v>0.08717118544798751</v>
       </c>
       <c r="F88">
-        <v>0.38232</v>
+        <v>0.3708504</v>
       </c>
       <c r="G88">
-        <v>0.08884759581220325</v>
+        <v>0.0888475958122032</v>
       </c>
       <c r="H88">
-        <v>0.38232</v>
+        <v>0.3937896</v>
       </c>
     </row>
     <row r="89" spans="1:8">
@@ -2697,19 +2697,19 @@
         <v>0.1037554984147873</v>
       </c>
       <c r="D89">
-        <v>0.42484</v>
+        <v>0.4503304</v>
       </c>
       <c r="E89">
-        <v>0.09207264659689611</v>
+        <v>0.0920726465968961</v>
       </c>
       <c r="F89">
-        <v>0.42484</v>
+        <v>0.4120948</v>
       </c>
       <c r="G89">
-        <v>0.09391791557386822</v>
+        <v>0.09391791557386819</v>
       </c>
       <c r="H89">
-        <v>0.42484</v>
+        <v>0.4375852</v>
       </c>
     </row>
     <row r="90" spans="1:8">
@@ -2723,19 +2723,19 @@
         <v>0.1103491570495166</v>
       </c>
       <c r="D90">
-        <v>0.47187</v>
+        <v>0.5001822</v>
       </c>
       <c r="E90">
-        <v>0.09748564543686719</v>
+        <v>0.09748564543686709</v>
       </c>
       <c r="F90">
-        <v>0.47187</v>
+        <v>0.4577139</v>
       </c>
       <c r="G90">
-        <v>0.09951739584196881</v>
+        <v>0.09951739584196879</v>
       </c>
       <c r="H90">
-        <v>0.47187</v>
+        <v>0.4860261</v>
       </c>
     </row>
     <row r="91" spans="1:8">
@@ -2749,19 +2749,19 @@
         <v>0.1177358674100725</v>
       </c>
       <c r="D91">
-        <v>0.52399</v>
+        <v>0.5554294</v>
       </c>
       <c r="E91">
         <v>0.1035496922472816</v>
       </c>
       <c r="F91">
-        <v>0.52399</v>
+        <v>0.5082703</v>
       </c>
       <c r="G91">
         <v>0.1057903531182602</v>
       </c>
       <c r="H91">
-        <v>0.52399</v>
+        <v>0.5397097</v>
       </c>
     </row>
     <row r="92" spans="1:8">
@@ -2775,19 +2775,19 @@
         <v>0.126368801911213</v>
       </c>
       <c r="D92">
-        <v>0.58201</v>
+        <v>0.6169306000000001</v>
       </c>
       <c r="E92">
         <v>0.110636814439821</v>
       </c>
       <c r="F92">
-        <v>0.58201</v>
+        <v>0.5645497</v>
       </c>
       <c r="G92">
         <v>0.1131216314074228</v>
       </c>
       <c r="H92">
-        <v>0.58201</v>
+        <v>0.5994703</v>
       </c>
     </row>
     <row r="93" spans="1:8">
@@ -2801,19 +2801,19 @@
         <v>0.1329398019252044</v>
       </c>
       <c r="D93">
-        <v>0.64741</v>
+        <v>0.6862546</v>
       </c>
       <c r="E93">
         <v>0.116031211909208</v>
       </c>
       <c r="F93">
-        <v>0.64741</v>
+        <v>0.6279877</v>
       </c>
       <c r="G93">
         <v>0.1187018694752894</v>
       </c>
       <c r="H93">
-        <v>0.64741</v>
+        <v>0.6668323</v>
       </c>
     </row>
     <row r="94" spans="1:8">
@@ -2827,19 +2827,19 @@
         <v>0.1433401088439011</v>
       </c>
       <c r="D94">
-        <v>0.7190800000000001</v>
+        <v>0.7622248000000001</v>
       </c>
       <c r="E94">
         <v>0.1245692410073068</v>
       </c>
       <c r="F94">
-        <v>0.7190800000000001</v>
+        <v>0.6975076</v>
       </c>
       <c r="G94">
         <v>0.1275340393827058</v>
       </c>
       <c r="H94">
-        <v>0.7190800000000001</v>
+        <v>0.7406524000000001</v>
       </c>
     </row>
     <row r="95" spans="1:8">
@@ -2853,19 +2853,19 @@
         <v>0.15350250024485</v>
       </c>
       <c r="D95">
-        <v>0.7996799999999999</v>
+        <v>0.8476608</v>
       </c>
       <c r="E95">
         <v>0.1329119557142725</v>
       </c>
       <c r="F95">
-        <v>0.7996799999999999</v>
+        <v>0.7756896</v>
       </c>
       <c r="G95">
-        <v>0.1361641661876649</v>
+        <v>0.1361641661876648</v>
       </c>
       <c r="H95">
-        <v>0.7996799999999999</v>
+        <v>0.8236703999999999</v>
       </c>
     </row>
     <row r="96" spans="1:8">
@@ -2876,22 +2876,22 @@
         <v>0.88997</v>
       </c>
       <c r="C96">
-        <v>0.1623167037118937</v>
+        <v>0.1623167037118936</v>
       </c>
       <c r="D96">
-        <v>0.88997</v>
+        <v>0.9433682000000001</v>
       </c>
       <c r="E96">
-        <v>0.1401478888714847</v>
+        <v>0.1401478888714846</v>
       </c>
       <c r="F96">
-        <v>0.88997</v>
+        <v>0.8632709000000001</v>
       </c>
       <c r="G96">
-        <v>0.1436493820786998</v>
+        <v>0.1436493820786997</v>
       </c>
       <c r="H96">
-        <v>0.88997</v>
+        <v>0.9166691</v>
       </c>
     </row>
     <row r="97" spans="1:8">
@@ -2905,19 +2905,19 @@
         <v>0.1730908778727658</v>
       </c>
       <c r="D97">
-        <v>0.99069</v>
+        <v>1.0501314</v>
       </c>
       <c r="E97">
         <v>0.148992840584221</v>
       </c>
       <c r="F97">
-        <v>0.99069</v>
+        <v>0.9609692999999999</v>
       </c>
       <c r="G97">
         <v>0.1527990482899775</v>
       </c>
       <c r="H97">
-        <v>0.99069</v>
+        <v>1.0204107</v>
       </c>
     </row>
     <row r="98" spans="1:8">
@@ -2928,22 +2928,22 @@
         <v>1.10018</v>
       </c>
       <c r="C98">
-        <v>0.1890765348033553</v>
+        <v>0.1890765348033552</v>
       </c>
       <c r="D98">
-        <v>1.10018</v>
+        <v>1.1661908</v>
       </c>
       <c r="E98">
         <v>0.1621161075312987</v>
       </c>
       <c r="F98">
-        <v>1.10018</v>
+        <v>1.0671746</v>
       </c>
       <c r="G98">
-        <v>0.1663744205550806</v>
+        <v>0.1663744205550805</v>
       </c>
       <c r="H98">
-        <v>1.10018</v>
+        <v>1.1331854</v>
       </c>
     </row>
     <row r="99" spans="1:8">
@@ -2954,22 +2954,22 @@
         <v>1.22296</v>
       </c>
       <c r="C99">
-        <v>0.2063084158745294</v>
+        <v>0.2063084158745293</v>
       </c>
       <c r="D99">
-        <v>1.22296</v>
+        <v>1.2963376</v>
       </c>
       <c r="E99">
-        <v>0.1762624498605015</v>
+        <v>0.1762624498605014</v>
       </c>
       <c r="F99">
-        <v>1.22296</v>
+        <v>1.1862712</v>
       </c>
       <c r="G99">
-        <v>0.1810081138330548</v>
+        <v>0.1810081138330547</v>
       </c>
       <c r="H99">
-        <v>1.22296</v>
+        <v>1.2596488</v>
       </c>
     </row>
     <row r="100" spans="1:8">
@@ -2983,19 +2983,19 @@
         <v>0.2069881744966664</v>
       </c>
       <c r="D100">
-        <v>1.36697</v>
+        <v>1.4489882</v>
       </c>
       <c r="E100">
         <v>0.1768204909780243</v>
       </c>
       <c r="F100">
-        <v>1.36697</v>
+        <v>1.3259609</v>
       </c>
       <c r="G100">
-        <v>0.1815853798400754</v>
+        <v>0.1815853798400753</v>
       </c>
       <c r="H100">
-        <v>1.36697</v>
+        <v>1.4079791</v>
       </c>
     </row>
     <row r="101" spans="1:8">
@@ -3009,19 +3009,19 @@
         <v>0.2356739883508497</v>
       </c>
       <c r="D101">
-        <v>1.51913</v>
+        <v>1.6102778</v>
       </c>
       <c r="E101">
-        <v>0.2003698261374862</v>
+        <v>0.2003698261374861</v>
       </c>
       <c r="F101">
-        <v>1.51913</v>
+        <v>1.4735561</v>
       </c>
       <c r="G101">
         <v>0.2059460053363481</v>
       </c>
       <c r="H101">
-        <v>1.51913</v>
+        <v>1.5647039</v>
       </c>
     </row>
     <row r="102" spans="1:8">
@@ -3035,19 +3035,19 @@
         <v>0.249620369415028</v>
       </c>
       <c r="D102">
-        <v>1.6984</v>
+        <v>1.800304</v>
       </c>
       <c r="E102">
-        <v>0.2118189697319955</v>
+        <v>0.2118189697319954</v>
       </c>
       <c r="F102">
-        <v>1.6984</v>
+        <v>1.647448</v>
       </c>
       <c r="G102">
         <v>0.217789579580389</v>
       </c>
       <c r="H102">
-        <v>1.6984</v>
+        <v>1.749352</v>
       </c>
     </row>
   </sheetData>

</xml_diff>